<commit_message>
Cleaned up and added data json objects for easy element access and manipulation
</commit_message>
<xml_diff>
--- a/src/pages/SampleMilestone.xlsx
+++ b/src/pages/SampleMilestone.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nigellim/Desktop/summerbuild-2025/src/pages/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89FF7787-CB77-604E-8EB0-C93022098A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D9271E-54EC-684D-B0C6-C38D33EFCDF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="500" windowWidth="16840" windowHeight="10400" xr2:uid="{6A960687-A5A5-1548-9F9D-356A824E6568}"/>
+    <workbookView xWindow="100" yWindow="500" windowWidth="38200" windowHeight="21000" xr2:uid="{6A960687-A5A5-1548-9F9D-356A824E6568}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="11">
   <si>
     <t>Team</t>
   </si>
@@ -47,22 +47,28 @@
     <t>Milestone2</t>
   </si>
   <si>
-    <t>Aloy</t>
-  </si>
-  <si>
     <t>Y</t>
   </si>
   <si>
-    <t>Maven</t>
-  </si>
-  <si>
     <t>N</t>
   </si>
   <si>
     <t>Milestone3</t>
   </si>
   <si>
-    <t>S</t>
+    <t>Team1</t>
+  </si>
+  <si>
+    <t>Team2</t>
+  </si>
+  <si>
+    <t>Milestone4</t>
+  </si>
+  <si>
+    <t>Milestone5</t>
+  </si>
+  <si>
+    <t>Team3</t>
   </si>
 </sst>
 </file>
@@ -434,10 +440,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3227CAED-1262-6F46-91EE-337667515699}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -448,35 +454,73 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>